<commit_message>
Agrega prospectos y documento de presentacion BarberAI
</commit_message>
<xml_diff>
--- a/prospectos/prospectos_barberai_comayagua.xlsx
+++ b/prospectos/prospectos_barberai_comayagua.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\landing-barberai\prospectos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CD12E52E-3C6B-441E-90AB-258939014D06}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A81322D4-75E0-4845-8C97-1AC04C32AA4B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="9525" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="128">
   <si>
     <t>Prospectos BarberAI - Comayagua</t>
   </si>
@@ -54,9 +54,6 @@
     <t>Fuente pública</t>
   </si>
   <si>
-    <t>Confianza del dato</t>
-  </si>
-  <si>
     <t>Owen Club Barber</t>
   </si>
   <si>
@@ -84,9 +81,6 @@
     <t>https://book.heygoldie.com/OWEN-CLUBBARBER</t>
   </si>
   <si>
-    <t>Alta</t>
-  </si>
-  <si>
     <t>É Cavaleiro</t>
   </si>
   <si>
@@ -172,9 +166,6 @@
   </si>
   <si>
     <t>https://www.instagram.com/0101barbershop_comayagua/</t>
-  </si>
-  <si>
-    <t>Media</t>
   </si>
   <si>
     <t>ISAI Barber Shop Comayagua</t>
@@ -532,8 +523,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProspectosTable" displayName="ProspectosTable" ref="A4:J19">
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProspectosTable" displayName="ProspectosTable" ref="A4:I19">
+  <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Nombre del negocio"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Ciudad/zona"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Teléfono/WhatsApp"/>
@@ -543,7 +534,6 @@
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Cómo BarberAI les ayudaría"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Estado"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Fuente pública"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Confianza del dato"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -766,488 +756,440 @@
       <c r="I4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="5" spans="1:10" ht="71.25">
       <c r="A5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="H5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="57">
       <c r="A6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="H6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="57">
       <c r="A7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="H7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="42.75">
       <c r="A8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="E8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="2" t="s">
+      <c r="H8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="42.75">
       <c r="A9" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="E9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" s="2" t="s">
+      <c r="H9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I9" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="42.75">
       <c r="A10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="H10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I10" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="28.5">
       <c r="A11" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D11" s="2" t="s">
+      <c r="H11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I11" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57">
       <c r="A12" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="H12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I12" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="42.75">
       <c r="A13" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C13" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="G13" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="H13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I13" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="28.5">
       <c r="A14" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="2" t="s">
+      <c r="F14" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="G14" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="H14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I14" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="28.5">
       <c r="A15" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="F15" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="H15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I15" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="28.5">
       <c r="A16" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="E16" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="G16" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="H16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I16" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="F16" s="2" t="s">
+    </row>
+    <row r="17" spans="1:9" ht="42.75">
+      <c r="A17" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="B17" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="H16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I16" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="J16" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="28.5">
-      <c r="A17" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C17" s="2" t="s">
+      <c r="F17" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="H17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I17" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="F17" s="2" t="s">
+    </row>
+    <row r="18" spans="1:9" ht="28.5">
+      <c r="A18" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="B18" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="H17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I17" s="2" t="s">
+      <c r="C18" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="J17" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="28.5">
-      <c r="A18" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="F18" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="G18" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="H18" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I18" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="F18" s="2" t="s">
+    </row>
+    <row r="19" spans="1:9" ht="71.25">
+      <c r="A19" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="B19" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="H18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I18" s="2" t="s">
+      <c r="D19" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="J18" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="71.25">
-      <c r="A19" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C19" s="2" t="s">
+      <c r="F19" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="G19" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="H19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I19" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1263,17 +1205,9 @@
       <formula>"Interesado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J5:J19">
-    <cfRule type="cellIs" priority="3">
-      <formula>"Media"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="1">
     <dataValidation type="list" sqref="H5:H19" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Pendiente,Contactado,Interesado,No interesado"</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="J5:J19" xr:uid="{00000000-0002-0000-0000-000001000000}">
-      <formula1>"Alta,Media,Baja"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1295,7 +1229,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="27.95" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -1305,15 +1239,15 @@
     </row>
     <row r="3" spans="1:6" ht="27.95" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="3" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B4" s="3">
         <v>15</v>
@@ -1321,39 +1255,39 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="3" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="3" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="3" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="3" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15">
       <c r="A10" s="7" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -1363,7 +1297,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="8" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>

</xml_diff>